<commit_message>
New data for December 2024
</commit_message>
<xml_diff>
--- a/AH2700A checks KJ.xlsx
+++ b/AH2700A checks KJ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callaghaninnovationgovtnz-my.sharepoint.com/personal/keith_jones_callaghaninnovation_govt_nz/Documents/KJ/PycharmProjects/CapacitanceScale/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="354" documentId="8_{94DDC3C1-F777-4C57-BE64-BE5D48C8AE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0814B75-9373-4E37-8E08-99BA0231F5C5}"/>
+  <xr:revisionPtr revIDLastSave="361" documentId="8_{94DDC3C1-F777-4C57-BE64-BE5D48C8AE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB8969E7-12A1-427D-9851-136F54A4F8F5}"/>
   <bookViews>
-    <workbookView xWindow="-28140" yWindow="900" windowWidth="27135" windowHeight="14100" tabRatio="835" firstSheet="21" activeTab="26" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23820" yWindow="1125" windowWidth="21600" windowHeight="11775" tabRatio="835" firstSheet="21" activeTab="28" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AH2700A2022-04-07" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,11 @@
     <sheet name="AH2700A2023-10-02" sheetId="27" r:id="rId23"/>
     <sheet name="AH2700A2023-12-18" sheetId="28" r:id="rId24"/>
     <sheet name="AH2700A2024-7-25" sheetId="29" r:id="rId25"/>
-    <sheet name="Checks" sheetId="3" r:id="rId26"/>
-    <sheet name="Summary" sheetId="20" r:id="rId27"/>
-    <sheet name="Conditions" sheetId="30" r:id="rId28"/>
-    <sheet name="KJ notes" sheetId="21" r:id="rId29"/>
+    <sheet name="Sheet1" sheetId="31" r:id="rId26"/>
+    <sheet name="Checks" sheetId="3" r:id="rId27"/>
+    <sheet name="Summary" sheetId="20" r:id="rId28"/>
+    <sheet name="Conditions" sheetId="30" r:id="rId29"/>
+    <sheet name="KJ notes" sheetId="21" r:id="rId30"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1428" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="240">
   <si>
     <t>av_exp = 10,   frequency = 1591.5,   no. of samples = 10,   settling samples = 2</t>
   </si>
@@ -766,6 +767,24 @@
   </si>
   <si>
     <t>Conlcude that 1000 pF b has likely shifted 2 ppm</t>
+  </si>
+  <si>
+    <t>Zero WITH BNC/BPO connectors 14:31 1010.10mbar, 52.24%RH 20.56C FCU011</t>
+  </si>
+  <si>
+    <t>AH11_1: 11.9, -11.6, 30.1, .036, -.019, -.014, .019</t>
+  </si>
+  <si>
+    <t>AH11_2: 11.8, -11.8, 29.6, -.055, -.071, -.032, .017</t>
+  </si>
+  <si>
+    <t>GR inner 23.9060, 1009.97mbar</t>
+  </si>
+  <si>
+    <t>Permuteable Temp 22.75(by GMH5I), setting of oil bath 23.000,</t>
+  </si>
+  <si>
+    <t>s-ball 23.735 GRinner 23.9055, GRouter 23.883;GMH5I 20.80 under UB cap, in S ball oil 23.32</t>
   </si>
 </sst>
 </file>
@@ -50181,6 +50200,1468 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A53FF85B-959F-4593-AC2F-7184A9E9A9F6}">
+  <dimension ref="A1:P30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N1">
+        <v>-4.2</v>
+      </c>
+      <c r="O1" t="s">
+        <v>4</v>
+      </c>
+      <c r="P1">
+        <f>N1 - N6</f>
+        <v>-2.339719999956654</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
+        <v>45637.604247233794</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="1">
+        <v>-1.2200000000000001E-7</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4.5343136195018498E-8</v>
+      </c>
+      <c r="E3" s="1">
+        <v>2.6800000000000001E-5</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1.4028542333400101E-6</v>
+      </c>
+      <c r="G3">
+        <v>1591.5</v>
+      </c>
+      <c r="H3">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>234</v>
+      </c>
+      <c r="J3">
+        <f>C3-C$3</f>
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <f>D3-D$3</f>
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
+        <v>45637.606466886573</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>9.9999765790000001</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1.11754194387178E-7</v>
+      </c>
+      <c r="E4">
+        <v>-1.6369999999999899E-4</v>
+      </c>
+      <c r="F4" s="1">
+        <v>9.0553851381374296E-7</v>
+      </c>
+      <c r="G4">
+        <v>1591.5</v>
+      </c>
+      <c r="H4">
+        <v>15</v>
+      </c>
+      <c r="I4" t="s">
+        <v>235</v>
+      </c>
+      <c r="J4">
+        <f t="shared" ref="J4:J30" si="0">C4-C$3</f>
+        <v>9.9999767009999996</v>
+      </c>
+      <c r="K4">
+        <f>E4-E$3</f>
+        <v>-1.9049999999999899E-4</v>
+      </c>
+      <c r="L4">
+        <f>K4*0.000000001/(2*PI()*J4*G4*0.000000000001)</f>
+        <v>-1.9050636066256616E-6</v>
+      </c>
+      <c r="M4">
+        <v>10</v>
+      </c>
+      <c r="N4">
+        <f>(J4/M4-1)*1000000</f>
+        <v>-2.3299000000420733</v>
+      </c>
+      <c r="O4">
+        <f>N4+P$1</f>
+        <v>-4.6696199999987273</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="9">
+        <v>45637.608341388892</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5">
+        <v>9.99997920499999</v>
+      </c>
+      <c r="D5" s="1">
+        <v>7.6190550720851104E-8</v>
+      </c>
+      <c r="E5">
+        <v>-1.3239999999999999E-4</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1.22147451876819E-6</v>
+      </c>
+      <c r="G5">
+        <v>1591.5</v>
+      </c>
+      <c r="H5">
+        <v>15</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>9.9999793269999895</v>
+      </c>
+      <c r="K5">
+        <f t="shared" ref="K5:K30" si="1">E5-E$3</f>
+        <v>-1.5919999999999999E-4</v>
+      </c>
+      <c r="L5">
+        <f t="shared" ref="L5:L30" si="2">K5*0.000000001/(2*PI()*J5*G5*0.000000000001)</f>
+        <v>-1.5920527376992432E-6</v>
+      </c>
+      <c r="M5">
+        <v>10</v>
+      </c>
+      <c r="N5">
+        <f t="shared" ref="N5:N30" si="3">(J5/M5-1)*1000000</f>
+        <v>-2.0673000010740239</v>
+      </c>
+      <c r="O5">
+        <f t="shared" ref="O5:O30" si="4">N5+P$1</f>
+        <v>-4.4070200010306779</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="9">
+        <v>45637.609701319445</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>99.999813849999995</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1.43178210569032E-7</v>
+      </c>
+      <c r="E6">
+        <v>1.9388999999999999E-3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>9.4339811320565396E-7</v>
+      </c>
+      <c r="G6">
+        <v>1591.5</v>
+      </c>
+      <c r="H6">
+        <v>15</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>99.999813971999998</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="1"/>
+        <v>1.9120999999999999E-3</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="2"/>
+        <v>1.912162945697681E-6</v>
+      </c>
+      <c r="M6">
+        <v>100</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="3"/>
+        <v>-1.8602800000433461</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="4"/>
+        <v>-4.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
+        <v>45637.610507361111</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7">
+        <v>99.99983014</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1.01980393135795E-7</v>
+      </c>
+      <c r="E7">
+        <v>2.2363999999999999E-3</v>
+      </c>
+      <c r="F7" s="1">
+        <v>3.0066592756745399E-6</v>
+      </c>
+      <c r="G7">
+        <v>1591.5</v>
+      </c>
+      <c r="H7">
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>99.999830262000003</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="1"/>
+        <v>2.2095999999999999E-3</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="2"/>
+        <v>2.2096723793426884E-6</v>
+      </c>
+      <c r="M7">
+        <v>100</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="3"/>
+        <v>-1.6973799999986383</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="4"/>
+        <v>-4.0370999999552923</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="9">
+        <v>45637.611628923609</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>9.9999776659999906</v>
+      </c>
+      <c r="D8" s="1">
+        <v>7.9271684790939105E-8</v>
+      </c>
+      <c r="E8">
+        <v>-2.7838E-4</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1.1762652762026E-6</v>
+      </c>
+      <c r="G8">
+        <v>1591.5</v>
+      </c>
+      <c r="H8">
+        <v>15</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="0"/>
+        <v>9.99997778799999</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="1"/>
+        <v>-3.0518E-4</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="2"/>
+        <v>-3.0519015657379626E-6</v>
+      </c>
+      <c r="M8">
+        <v>10</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="3"/>
+        <v>-2.2212000010402022</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="4"/>
+        <v>-4.5609200009968562</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="9">
+        <v>45637.612543900461</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9">
+        <v>9.9999753869999992</v>
+      </c>
+      <c r="D9" s="1">
+        <v>8.4504437684310093E-8</v>
+      </c>
+      <c r="E9">
+        <v>-2.2468999999999999E-4</v>
+      </c>
+      <c r="F9" s="1">
+        <v>8.7914731416299103E-7</v>
+      </c>
+      <c r="G9">
+        <v>1591.5</v>
+      </c>
+      <c r="H9">
+        <v>15</v>
+      </c>
+      <c r="I9" t="s">
+        <v>236</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="0"/>
+        <v>9.9999755089999987</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="1"/>
+        <v>-2.5148999999999999E-4</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="2"/>
+        <v>-2.514984270549502E-6</v>
+      </c>
+      <c r="M9">
+        <v>10</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="3"/>
+        <v>-2.4491000001347629</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="4"/>
+        <v>-4.788820000091417</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="9">
+        <v>45637.613870196757</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10">
+        <v>99.999802090000003</v>
+      </c>
+      <c r="D10" s="1">
+        <v>9.4339810540097306E-8</v>
+      </c>
+      <c r="E10">
+        <v>8.5429999999999903E-4</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1.00498756211206E-6</v>
+      </c>
+      <c r="G10">
+        <v>1591.5</v>
+      </c>
+      <c r="H10">
+        <v>15</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="0"/>
+        <v>99.999802212000006</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="1"/>
+        <v>8.2749999999999903E-4</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="2"/>
+        <v>8.2752733834288071E-7</v>
+      </c>
+      <c r="M10">
+        <v>100</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="3"/>
+        <v>-1.9778799998926289</v>
+      </c>
+      <c r="O10">
+        <f t="shared" si="4"/>
+        <v>-4.3175999998492829</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="9">
+        <v>45637.614799143521</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11">
+        <v>99.999890539999996</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1.1999999737592299E-7</v>
+      </c>
+      <c r="E11">
+        <v>9.3619999999999999E-4</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1.32664991614217E-6</v>
+      </c>
+      <c r="G11">
+        <v>1591.5</v>
+      </c>
+      <c r="H11">
+        <v>15</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="0"/>
+        <v>99.999890661999999</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="1"/>
+        <v>9.0939999999999999E-4</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="2"/>
+        <v>9.0942923970373467E-7</v>
+      </c>
+      <c r="M11">
+        <v>100</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="3"/>
+        <v>-1.0933799999834903</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="4"/>
+        <v>-3.4330999999401444</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="9">
+        <v>45637.631125231484</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12">
+        <v>10.000194689999899</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1.37477271046848E-7</v>
+      </c>
+      <c r="E12">
+        <v>9.4844999999999999E-4</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1.3887044321957001E-6</v>
+      </c>
+      <c r="G12">
+        <v>1591.5</v>
+      </c>
+      <c r="H12">
+        <v>15</v>
+      </c>
+      <c r="I12" t="s">
+        <v>237</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="0"/>
+        <v>10.000194811999899</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="1"/>
+        <v>9.2164999999999999E-4</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="2"/>
+        <v>9.2166067077289861E-6</v>
+      </c>
+      <c r="M12">
+        <v>10</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="3"/>
+        <v>19.481199989845877</v>
+      </c>
+      <c r="O12">
+        <f t="shared" si="4"/>
+        <v>17.141479989889223</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="9">
+        <v>45637.632679270835</v>
+      </c>
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13">
+        <v>100.00412900000001</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>8.6301999999999993E-3</v>
+      </c>
+      <c r="F13" s="1">
+        <v>2.7294688127912899E-6</v>
+      </c>
+      <c r="G13">
+        <v>1591.5</v>
+      </c>
+      <c r="H13">
+        <v>15</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="0"/>
+        <v>100.00412912200001</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="1"/>
+        <v>8.6033999999999989E-3</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="2"/>
+        <v>8.6033119745666183E-6</v>
+      </c>
+      <c r="M13">
+        <v>100</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="3"/>
+        <v>41.29122000007257</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="4"/>
+        <v>38.951500000115914</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="9">
+        <v>45637.668966296296</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14">
+        <v>1000.032592</v>
+      </c>
+      <c r="D14" s="1">
+        <v>3.99999998990097E-6</v>
+      </c>
+      <c r="E14">
+        <v>0.195855</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2.6925824035674102E-5</v>
+      </c>
+      <c r="G14">
+        <v>1591.5</v>
+      </c>
+      <c r="H14">
+        <v>1.5</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="0"/>
+        <v>1000.032592122</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="1"/>
+        <v>0.19582820000000001</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="2"/>
+        <v>1.9582789984530093E-5</v>
+      </c>
+      <c r="M14">
+        <v>1000</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="3"/>
+        <v>32.59212199990813</v>
+      </c>
+      <c r="O14">
+        <f t="shared" si="4"/>
+        <v>30.252401999951477</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
+        <v>45637.670517372688</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15">
+        <v>1000.003</v>
+      </c>
+      <c r="D15">
+        <v>1.8132843129675999E-4</v>
+      </c>
+      <c r="E15">
+        <v>0.210034</v>
+      </c>
+      <c r="F15">
+        <v>2.6792536274119902E-4</v>
+      </c>
+      <c r="G15">
+        <v>1591.5</v>
+      </c>
+      <c r="H15">
+        <v>1.5</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="0"/>
+        <v>1000.003000122</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="1"/>
+        <v>0.2100072</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="2"/>
+        <v>2.1001309261740207E-5</v>
+      </c>
+      <c r="M15">
+        <v>1000</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="3"/>
+        <v>3.0001219999409301</v>
+      </c>
+      <c r="O15">
+        <f t="shared" si="4"/>
+        <v>0.66040199998427607</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="9">
+        <v>45637.672379791664</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16">
+        <v>4.9999502749999998</v>
+      </c>
+      <c r="D16" s="1">
+        <v>6.0868711256547894E-8</v>
+      </c>
+      <c r="E16">
+        <v>2.5175000000000002E-4</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1.68300326797068E-6</v>
+      </c>
+      <c r="G16">
+        <v>1591.5</v>
+      </c>
+      <c r="H16">
+        <v>15</v>
+      </c>
+      <c r="I16" t="s">
+        <v>238</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="0"/>
+        <v>4.9999503970000001</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="1"/>
+        <v>2.2495000000000002E-4</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="2"/>
+        <v>4.4991843705207329E-6</v>
+      </c>
+      <c r="M16">
+        <v>5</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="3"/>
+        <v>-9.9205999999352201</v>
+      </c>
+      <c r="O16">
+        <f t="shared" si="4"/>
+        <v>-12.260319999891873</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="9">
+        <v>45637.673785416664</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17">
+        <v>5.000107979</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2.5664956646134801E-7</v>
+      </c>
+      <c r="E17" s="1">
+        <v>-5.4819999999999899E-5</v>
+      </c>
+      <c r="F17" s="1">
+        <v>8.40358709123669E-5</v>
+      </c>
+      <c r="G17">
+        <v>1591.5</v>
+      </c>
+      <c r="H17">
+        <v>15</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="0"/>
+        <v>5.0001081010000004</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="1"/>
+        <v>-8.16199999999999E-5</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="2"/>
+        <v>-1.6324154080978203E-6</v>
+      </c>
+      <c r="M17">
+        <v>5</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="3"/>
+        <v>21.620200000072032</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="4"/>
+        <v>19.280480000115379</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="9">
+        <v>45637.675926898148</v>
+      </c>
+      <c r="B18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18">
+        <v>0.50005215999999997</v>
+      </c>
+      <c r="D18" s="1">
+        <v>6.8992753246556301E-8</v>
+      </c>
+      <c r="E18" s="1">
+        <v>7.9799999999999893E-5</v>
+      </c>
+      <c r="F18" s="1">
+        <v>9.5812316536027895E-7</v>
+      </c>
+      <c r="G18">
+        <v>1591.5</v>
+      </c>
+      <c r="H18">
+        <v>15</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="0"/>
+        <v>0.50005228199999996</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="1"/>
+        <v>5.2999999999999892E-5</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="2"/>
+        <v>1.0599220931928874E-5</v>
+      </c>
+      <c r="M18">
+        <v>0.5</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="3"/>
+        <v>104.56399999991817</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="4"/>
+        <v>102.22427999996151</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="9">
+        <v>45637.679648101854</v>
+      </c>
+      <c r="B19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19">
+        <v>1000.162698</v>
+      </c>
+      <c r="D19">
+        <v>1.09708705218229E-4</v>
+      </c>
+      <c r="E19">
+        <v>1.1263300000000001</v>
+      </c>
+      <c r="F19">
+        <v>0.68349651067141504</v>
+      </c>
+      <c r="G19">
+        <v>1591.5</v>
+      </c>
+      <c r="H19">
+        <v>1.5</v>
+      </c>
+      <c r="I19" t="s">
+        <v>239</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="0"/>
+        <v>1000.1626981219999</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="1"/>
+        <v>1.1263031999999999</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="2"/>
+        <v>1.1261549589225157E-4</v>
+      </c>
+      <c r="M19">
+        <v>1000</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="3"/>
+        <v>162.69812199998233</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="4"/>
+        <v>160.35840200002568</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="9">
+        <v>45637.685070671294</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20">
+        <v>10.00040811</v>
+      </c>
+      <c r="D20" s="1">
+        <v>9.4339811443904304E-8</v>
+      </c>
+      <c r="E20">
+        <v>4.8140999999999999E-4</v>
+      </c>
+      <c r="F20" s="1">
+        <v>1.46318146516418E-6</v>
+      </c>
+      <c r="G20">
+        <v>1591.5</v>
+      </c>
+      <c r="H20">
+        <v>15</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="0"/>
+        <v>10.000408232</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="1"/>
+        <v>4.5460999999999999E-4</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="2"/>
+        <v>4.5460556142690165E-6</v>
+      </c>
+      <c r="M20">
+        <v>10</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="3"/>
+        <v>40.823199999984183</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="4"/>
+        <v>38.483480000027527</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="9">
+        <v>45637.688239201387</v>
+      </c>
+      <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21">
+        <v>10.00015973</v>
+      </c>
+      <c r="D21" s="1">
+        <v>1.18743420971498E-7</v>
+      </c>
+      <c r="E21">
+        <v>4.7926999999999898E-4</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1.20253898065717E-6</v>
+      </c>
+      <c r="G21">
+        <v>1591.5</v>
+      </c>
+      <c r="H21">
+        <v>15</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="0"/>
+        <v>10.000159851999999</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="1"/>
+        <v>4.5246999999999898E-4</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="2"/>
+        <v>4.5247682048122535E-6</v>
+      </c>
+      <c r="M21">
+        <v>10</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="3"/>
+        <v>15.985199999901667</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="4"/>
+        <v>13.645479999945014</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="9">
+        <v>45637.689535092592</v>
+      </c>
+      <c r="B22" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22">
+        <v>10.000127839999999</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.3564659954527201E-7</v>
+      </c>
+      <c r="E22">
+        <v>4.7107999999999899E-4</v>
+      </c>
+      <c r="F22" s="1">
+        <v>9.6726418314750192E-7</v>
+      </c>
+      <c r="G22">
+        <v>1591.5</v>
+      </c>
+      <c r="H22">
+        <v>15</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="0"/>
+        <v>10.000127961999999</v>
+      </c>
+      <c r="K22">
+        <f t="shared" si="1"/>
+        <v>4.4427999999999899E-4</v>
+      </c>
+      <c r="L22">
+        <f t="shared" si="2"/>
+        <v>4.4428811383824551E-6</v>
+      </c>
+      <c r="M22">
+        <v>10</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="3"/>
+        <v>12.796199999831614</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="4"/>
+        <v>10.456479999874961</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="9">
+        <v>45637.69070846065</v>
+      </c>
+      <c r="B23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23">
+        <v>10.000235729999901</v>
+      </c>
+      <c r="D23" s="1">
+        <v>1.3453624072258499E-7</v>
+      </c>
+      <c r="E23">
+        <v>5.0416999999999997E-4</v>
+      </c>
+      <c r="F23" s="1">
+        <v>1.2522379965485801E-6</v>
+      </c>
+      <c r="G23">
+        <v>1591.5</v>
+      </c>
+      <c r="H23">
+        <v>15</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="0"/>
+        <v>10.0002358519999</v>
+      </c>
+      <c r="K23">
+        <f t="shared" si="1"/>
+        <v>4.7736999999999996E-4</v>
+      </c>
+      <c r="L23">
+        <f t="shared" si="2"/>
+        <v>4.7737356783987244E-6</v>
+      </c>
+      <c r="M23">
+        <v>10</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="3"/>
+        <v>23.585199989906158</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="4"/>
+        <v>21.245479989949505</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="9">
+        <v>45637.691561122687</v>
+      </c>
+      <c r="B24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24">
+        <v>9.9999840019999997</v>
+      </c>
+      <c r="D24" s="1">
+        <v>1.34298175698956E-7</v>
+      </c>
+      <c r="E24">
+        <v>4.6921999999999898E-4</v>
+      </c>
+      <c r="F24" s="1">
+        <v>1.3399999999999899E-6</v>
+      </c>
+      <c r="G24">
+        <v>1591.5</v>
+      </c>
+      <c r="H24">
+        <v>15</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="0"/>
+        <v>9.9999841239999991</v>
+      </c>
+      <c r="K24">
+        <f t="shared" si="1"/>
+        <v>4.4241999999999898E-4</v>
+      </c>
+      <c r="L24">
+        <f t="shared" si="2"/>
+        <v>4.4243444367638229E-6</v>
+      </c>
+      <c r="M24">
+        <v>10</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="3"/>
+        <v>-1.5876000001302515</v>
+      </c>
+      <c r="O24">
+        <f t="shared" si="4"/>
+        <v>-3.9273200000869055</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="9">
+        <v>45637.692440833336</v>
+      </c>
+      <c r="B25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25">
+        <v>10.000243040000001</v>
+      </c>
+      <c r="D25" s="1">
+        <v>1.4282856844903899E-7</v>
+      </c>
+      <c r="E25">
+        <v>5.042E-4</v>
+      </c>
+      <c r="F25" s="1">
+        <v>7.4833147735480605E-7</v>
+      </c>
+      <c r="G25">
+        <v>1591.5</v>
+      </c>
+      <c r="H25">
+        <v>15</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="0"/>
+        <v>10.000243162</v>
+      </c>
+      <c r="K25">
+        <f t="shared" si="1"/>
+        <v>4.774E-4</v>
+      </c>
+      <c r="L25">
+        <f t="shared" si="2"/>
+        <v>4.7740321909056371E-6</v>
+      </c>
+      <c r="M25">
+        <v>10</v>
+      </c>
+      <c r="N25">
+        <f t="shared" si="3"/>
+        <v>24.316199999985244</v>
+      </c>
+      <c r="O25">
+        <f t="shared" si="4"/>
+        <v>21.976480000028591</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="9">
+        <v>45637.69359570602</v>
+      </c>
+      <c r="B26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26">
+        <v>10.0003471699999</v>
+      </c>
+      <c r="D26" s="1">
+        <v>1.7349351600561E-7</v>
+      </c>
+      <c r="E26">
+        <v>4.9595999999999896E-4</v>
+      </c>
+      <c r="F26" s="1">
+        <v>1.4256226709757199E-6</v>
+      </c>
+      <c r="G26">
+        <v>1591.5</v>
+      </c>
+      <c r="H26">
+        <v>15</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="0"/>
+        <v>10.000347291999899</v>
+      </c>
+      <c r="K26">
+        <f t="shared" si="1"/>
+        <v>4.6915999999999896E-4</v>
+      </c>
+      <c r="L26">
+        <f t="shared" si="2"/>
+        <v>4.6915827830218992E-6</v>
+      </c>
+      <c r="M26">
+        <v>10</v>
+      </c>
+      <c r="N26">
+        <f t="shared" si="3"/>
+        <v>34.729199990035653</v>
+      </c>
+      <c r="O26">
+        <f t="shared" si="4"/>
+        <v>32.389479990078996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="9">
+        <v>45637.694689467593</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27">
+        <v>10.00026188</v>
+      </c>
+      <c r="D27" s="1">
+        <v>1.46969384640714E-7</v>
+      </c>
+      <c r="E27">
+        <v>4.9516000000000002E-4</v>
+      </c>
+      <c r="F27" s="1">
+        <v>1.64450600485375E-6</v>
+      </c>
+      <c r="G27">
+        <v>1591.5</v>
+      </c>
+      <c r="H27">
+        <v>15</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="0"/>
+        <v>10.000262001999999</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="1"/>
+        <v>4.6836000000000002E-4</v>
+      </c>
+      <c r="L27">
+        <f t="shared" si="2"/>
+        <v>4.6836227576110604E-6</v>
+      </c>
+      <c r="M27">
+        <v>10</v>
+      </c>
+      <c r="N27">
+        <f t="shared" si="3"/>
+        <v>26.20019999999279</v>
+      </c>
+      <c r="O27">
+        <f t="shared" si="4"/>
+        <v>23.860480000036137</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="9">
+        <v>45637.696016504633</v>
+      </c>
+      <c r="B28" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28">
+        <v>10.00039568</v>
+      </c>
+      <c r="D28" s="1">
+        <v>9.7979589877313302E-8</v>
+      </c>
+      <c r="E28">
+        <v>5.0283999999999995E-4</v>
+      </c>
+      <c r="F28" s="1">
+        <v>1.2870120434557E-6</v>
+      </c>
+      <c r="G28">
+        <v>1591.5</v>
+      </c>
+      <c r="H28">
+        <v>15</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="0"/>
+        <v>10.000395802</v>
+      </c>
+      <c r="K28">
+        <f t="shared" si="1"/>
+        <v>4.7603999999999995E-4</v>
+      </c>
+      <c r="L28">
+        <f t="shared" si="2"/>
+        <v>4.7603594388416871E-6</v>
+      </c>
+      <c r="M28">
+        <v>10</v>
+      </c>
+      <c r="N28">
+        <f t="shared" si="3"/>
+        <v>39.580199999944554</v>
+      </c>
+      <c r="O28">
+        <f t="shared" si="4"/>
+        <v>37.240479999987897</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="9">
+        <v>45637.697016446757</v>
+      </c>
+      <c r="B29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29">
+        <v>10.00042</v>
+      </c>
+      <c r="D29" s="1">
+        <v>8.9442718556406002E-8</v>
+      </c>
+      <c r="E29">
+        <v>4.8888000000000002E-4</v>
+      </c>
+      <c r="F29" s="1">
+        <v>1.6277591959500701E-6</v>
+      </c>
+      <c r="G29">
+        <v>1591.5</v>
+      </c>
+      <c r="H29">
+        <v>15</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="0"/>
+        <v>10.000420122</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="1"/>
+        <v>4.6208000000000002E-4</v>
+      </c>
+      <c r="L29">
+        <f t="shared" si="2"/>
+        <v>4.6207493910907297E-6</v>
+      </c>
+      <c r="M29">
+        <v>10</v>
+      </c>
+      <c r="N29">
+        <f t="shared" si="3"/>
+        <v>42.012199999996724</v>
+      </c>
+      <c r="O29">
+        <f t="shared" si="4"/>
+        <v>39.672480000040068</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" s="9">
+        <v>45637.697994224538</v>
+      </c>
+      <c r="B30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30">
+        <v>10.000234749999899</v>
+      </c>
+      <c r="D30" s="1">
+        <v>1.11803398592713E-7</v>
+      </c>
+      <c r="E30">
+        <v>4.8819999999999999E-4</v>
+      </c>
+      <c r="F30" s="1">
+        <v>1.16533257055657E-6</v>
+      </c>
+      <c r="G30">
+        <v>1591.5</v>
+      </c>
+      <c r="H30">
+        <v>15</v>
+      </c>
+      <c r="I30" t="s">
+        <v>203</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="0"/>
+        <v>10.000234871999899</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="1"/>
+        <v>4.6139999999999999E-4</v>
+      </c>
+      <c r="L30">
+        <f t="shared" si="2"/>
+        <v>4.6140349369735491E-6</v>
+      </c>
+      <c r="M30">
+        <v>10</v>
+      </c>
+      <c r="N30">
+        <f t="shared" si="3"/>
+        <v>23.487199989791208</v>
+      </c>
+      <c r="O30">
+        <f t="shared" si="4"/>
+        <v>21.147479989834554</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3C34984-8EC3-4FA3-BF2E-2A86F7028EDB}">
   <dimension ref="A1:AH33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -53538,7 +55019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{156208CC-1640-424E-8C3D-7ABD6AEA3BA5}">
   <dimension ref="A1:AL103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -60025,7 +61506,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6523521-08A8-4AA4-9BC6-34BBF4C5CD24}">
   <dimension ref="D2:G28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -60396,65 +61877,22 @@
       </c>
     </row>
     <row r="28" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D28" s="6"/>
+      <c r="D28" s="6">
+        <v>45637</v>
+      </c>
+      <c r="E28">
+        <v>1009.97</v>
+      </c>
+      <c r="F28">
+        <v>23.905999999999999</v>
+      </c>
+      <c r="G28">
+        <v>23.9055</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{397F4A7E-BA8E-43E3-9CA2-FA7EC8F3CD27}">
-  <dimension ref="A2:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>227</v>
-      </c>
-      <c r="E5" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="21">
-        <v>5.8690000000000001E-4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>230</v>
-      </c>
-      <c r="G8" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>233</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -61381,6 +62819,60 @@
       <c r="O19" s="5">
         <f t="shared" si="4"/>
         <v>147.40925799007076</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{397F4A7E-BA8E-43E3-9CA2-FA7EC8F3CD27}">
+  <dimension ref="A2:G13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>227</v>
+      </c>
+      <c r="E5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="21">
+        <v>5.8690000000000001E-4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>230</v>
+      </c>
+      <c r="G8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tidying code, more plots.
</commit_message>
<xml_diff>
--- a/AH2700A checks KJ.xlsx
+++ b/AH2700A checks KJ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callaghaninnovationgovtnz-my.sharepoint.com/personal/keith_jones_callaghaninnovation_govt_nz/Documents/KJ/PycharmProjects/CapacitanceScale/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="361" documentId="8_{94DDC3C1-F777-4C57-BE64-BE5D48C8AE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB8969E7-12A1-427D-9851-136F54A4F8F5}"/>
+  <xr:revisionPtr revIDLastSave="409" documentId="8_{94DDC3C1-F777-4C57-BE64-BE5D48C8AE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BB02CE3-65F7-45C0-8371-5195869A1A4F}"/>
   <bookViews>
-    <workbookView xWindow="-23820" yWindow="1125" windowWidth="21600" windowHeight="11775" tabRatio="835" firstSheet="21" activeTab="28" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2610" yWindow="1380" windowWidth="21600" windowHeight="11775" tabRatio="835" firstSheet="21" activeTab="28" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AH2700A2022-04-07" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
     <sheet name="AH2700A2023-10-02" sheetId="27" r:id="rId23"/>
     <sheet name="AH2700A2023-12-18" sheetId="28" r:id="rId24"/>
     <sheet name="AH2700A2024-7-25" sheetId="29" r:id="rId25"/>
-    <sheet name="Sheet1" sheetId="31" r:id="rId26"/>
+    <sheet name="AH2700A2024-12-11" sheetId="31" r:id="rId26"/>
     <sheet name="Checks" sheetId="3" r:id="rId27"/>
     <sheet name="Summary" sheetId="20" r:id="rId28"/>
     <sheet name="Conditions" sheetId="30" r:id="rId29"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="242">
   <si>
     <t>av_exp = 10,   frequency = 1591.5,   no. of samples = 10,   settling samples = 2</t>
   </si>
@@ -785,6 +785,12 @@
   </si>
   <si>
     <t>s-ball 23.735 GRinner 23.9055, GRouter 23.883;GMH5I 20.80 under UB cap, in S ball oil 23.32</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>UB</t>
   </si>
 </sst>
 </file>
@@ -61508,14 +61514,14 @@
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6523521-08A8-4AA4-9BC6-34BBF4C5CD24}">
-  <dimension ref="D2:G28"/>
+  <dimension ref="D2:I28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="13.5703125" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
         <v>207</v>
       </c>
@@ -61528,8 +61534,14 @@
       <c r="G2" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="3" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>240</v>
+      </c>
+      <c r="I2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="3" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D3" s="6">
         <v>44658</v>
       </c>
@@ -61539,8 +61551,14 @@
       <c r="F3">
         <v>25.46</v>
       </c>
-    </row>
-    <row r="4" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H3">
+        <v>23.33</v>
+      </c>
+      <c r="I3">
+        <v>21.09</v>
+      </c>
+    </row>
+    <row r="4" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D4" s="6">
         <v>44662</v>
       </c>
@@ -61553,8 +61571,14 @@
       <c r="G4">
         <v>23.295000000000002</v>
       </c>
-    </row>
-    <row r="5" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H4">
+        <v>23.34</v>
+      </c>
+      <c r="I4">
+        <v>20.72</v>
+      </c>
+    </row>
+    <row r="5" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D5" s="6">
         <v>44711</v>
       </c>
@@ -61567,8 +61591,11 @@
       <c r="G5">
         <v>21.655000000000001</v>
       </c>
-    </row>
-    <row r="6" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="I5">
+        <v>20.68</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D6" s="6">
         <v>44712</v>
       </c>
@@ -61581,8 +61608,11 @@
       <c r="G6">
         <v>23.658999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="I6">
+        <v>20.79</v>
+      </c>
+    </row>
+    <row r="7" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D7" s="6">
         <v>44714</v>
       </c>
@@ -61595,8 +61625,11 @@
       <c r="G7">
         <v>23.35</v>
       </c>
-    </row>
-    <row r="8" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>20.76</v>
+      </c>
+    </row>
+    <row r="8" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D8" s="6">
         <v>44732</v>
       </c>
@@ -61609,8 +61642,14 @@
       <c r="G8">
         <v>23.678000000000001</v>
       </c>
-    </row>
-    <row r="9" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H8">
+        <v>21</v>
+      </c>
+      <c r="I8">
+        <v>20.88</v>
+      </c>
+    </row>
+    <row r="9" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D9" s="6">
         <v>44733</v>
       </c>
@@ -61623,8 +61662,14 @@
       <c r="G9">
         <v>23.37</v>
       </c>
-    </row>
-    <row r="10" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H9">
+        <v>21.54</v>
+      </c>
+      <c r="I9">
+        <v>20.81</v>
+      </c>
+    </row>
+    <row r="10" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D10" s="6">
         <v>44733</v>
       </c>
@@ -61637,8 +61682,14 @@
       <c r="G10">
         <v>23.679400000000001</v>
       </c>
-    </row>
-    <row r="11" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H10">
+        <v>21.54</v>
+      </c>
+      <c r="I10">
+        <v>20.84</v>
+      </c>
+    </row>
+    <row r="11" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D11" s="6">
         <v>44746</v>
       </c>
@@ -61651,8 +61702,14 @@
       <c r="G11">
         <v>23.6843</v>
       </c>
-    </row>
-    <row r="12" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H11">
+        <v>21.5</v>
+      </c>
+      <c r="I11">
+        <v>20.74</v>
+      </c>
+    </row>
+    <row r="12" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D12" s="6">
         <v>44753</v>
       </c>
@@ -61665,8 +61722,14 @@
       <c r="G12">
         <v>23.686</v>
       </c>
-    </row>
-    <row r="13" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H12">
+        <v>21.8</v>
+      </c>
+      <c r="I12">
+        <v>21.03</v>
+      </c>
+    </row>
+    <row r="13" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D13" s="6">
         <v>44767</v>
       </c>
@@ -61679,8 +61742,14 @@
       <c r="G13">
         <v>23.686499999999999</v>
       </c>
-    </row>
-    <row r="14" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H13">
+        <v>21.5</v>
+      </c>
+      <c r="I13">
+        <v>20.89</v>
+      </c>
+    </row>
+    <row r="14" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D14" s="6">
         <v>44774</v>
       </c>
@@ -61693,8 +61762,14 @@
       <c r="G14">
         <v>23.78</v>
       </c>
-    </row>
-    <row r="15" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H14">
+        <v>21.62</v>
+      </c>
+      <c r="I14">
+        <v>20.86</v>
+      </c>
+    </row>
+    <row r="15" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D15" s="6">
         <v>44827</v>
       </c>
@@ -61707,8 +61782,14 @@
       <c r="G15">
         <v>23.686499999999999</v>
       </c>
-    </row>
-    <row r="16" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H15">
+        <v>21.69</v>
+      </c>
+      <c r="I15">
+        <v>20.89</v>
+      </c>
+    </row>
+    <row r="16" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D16" s="6">
         <v>44859</v>
       </c>
@@ -61721,8 +61802,14 @@
       <c r="G16">
         <v>23.786000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H16">
+        <v>21.6</v>
+      </c>
+      <c r="I16">
+        <v>20.71</v>
+      </c>
+    </row>
+    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D17" s="6">
         <v>44876</v>
       </c>
@@ -61735,8 +61822,14 @@
       <c r="G17">
         <v>24.757000000000001</v>
       </c>
-    </row>
-    <row r="18" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H17">
+        <v>21.5</v>
+      </c>
+      <c r="I17">
+        <v>20.77</v>
+      </c>
+    </row>
+    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D18" s="6">
         <v>44942</v>
       </c>
@@ -61749,8 +61842,14 @@
       <c r="G18">
         <v>24.757000000000001</v>
       </c>
-    </row>
-    <row r="19" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H18">
+        <v>21.56</v>
+      </c>
+      <c r="I18">
+        <v>20.74</v>
+      </c>
+    </row>
+    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D19" s="6">
         <v>45013</v>
       </c>
@@ -61763,8 +61862,11 @@
       <c r="G19">
         <v>23.733000000000001</v>
       </c>
-    </row>
-    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H19">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D20" s="6">
         <v>45054</v>
       </c>
@@ -61777,8 +61879,14 @@
       <c r="G20">
         <v>23.73</v>
       </c>
-    </row>
-    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H20">
+        <v>21.56</v>
+      </c>
+      <c r="I20">
+        <v>20.72</v>
+      </c>
+    </row>
+    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D21" s="6">
         <v>45062</v>
       </c>
@@ -61791,8 +61899,14 @@
       <c r="G21">
         <v>23.73</v>
       </c>
-    </row>
-    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H21">
+        <v>20.76</v>
+      </c>
+      <c r="I21">
+        <v>21.67</v>
+      </c>
+    </row>
+    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D22" s="6">
         <v>45063</v>
       </c>
@@ -61805,8 +61919,14 @@
       <c r="G22">
         <v>23.734000000000002</v>
       </c>
-    </row>
-    <row r="23" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H22">
+        <v>22.75</v>
+      </c>
+      <c r="I22">
+        <v>21.65</v>
+      </c>
+    </row>
+    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D23" s="6">
         <v>45069</v>
       </c>
@@ -61819,8 +61939,14 @@
       <c r="G23">
         <v>23.73</v>
       </c>
-    </row>
-    <row r="24" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H23">
+        <v>23.73</v>
+      </c>
+      <c r="I23">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D24" s="6">
         <v>45198</v>
       </c>
@@ -61833,8 +61959,11 @@
       <c r="G24">
         <v>23.73</v>
       </c>
-    </row>
-    <row r="25" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="I24">
+        <v>21.36</v>
+      </c>
+    </row>
+    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D25" s="6">
         <v>45201</v>
       </c>
@@ -61848,7 +61977,7 @@
         <v>23.738</v>
       </c>
     </row>
-    <row r="26" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D26" s="6">
         <v>45278</v>
       </c>
@@ -61861,8 +61990,14 @@
       <c r="G26">
         <v>23.727</v>
       </c>
-    </row>
-    <row r="27" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H26">
+        <v>22.76</v>
+      </c>
+      <c r="I26">
+        <v>20.94</v>
+      </c>
+    </row>
+    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D27" s="6">
         <v>45498</v>
       </c>
@@ -61875,8 +62010,14 @@
       <c r="G27">
         <v>23.73</v>
       </c>
-    </row>
-    <row r="28" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H27">
+        <v>22.76</v>
+      </c>
+      <c r="I27">
+        <v>20.88</v>
+      </c>
+    </row>
+    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D28" s="6">
         <v>45637</v>
       </c>
@@ -61888,6 +62029,12 @@
       </c>
       <c r="G28">
         <v>23.9055</v>
+      </c>
+      <c r="H28">
+        <v>22.75</v>
+      </c>
+      <c r="I28">
+        <v>20.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>